<commit_message>
Adjust <result.xlsx> with sorting and averaging.
</commit_message>
<xml_diff>
--- a/resource/result.xlsx
+++ b/resource/result.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b1fc4107772a6185/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_Files\_Lessons\ALGORITHM\Project\resource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{5BFC3DE5-5D6D-421B-964B-B7DC593EE6E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6B9FAC1-3667-4000-84A6-A9AE6DB45EE1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14622D44-2112-4698-B9D1-C7263E7E6A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EXACT" sheetId="9" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
   <si>
     <t>att48</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -161,10 +161,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>p15</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>pa561</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -230,7 +226,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Average Ratio</t>
+    <t>Average</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ratio</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -612,35 +612,35 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G1" s="5"/>
       <c r="H1" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I1" s="5"/>
       <c r="J1" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>5</v>
@@ -661,7 +661,7 @@
         <v>6</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -728,7 +728,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" s="2">
         <v>71</v>
@@ -785,7 +785,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{260DB66E-1FFD-4D32-BA5D-DB6972467A37}">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" style="1" customWidth="1"/>
@@ -795,7 +795,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>4</v>
@@ -835,562 +835,562 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B3" s="2">
-        <v>2579</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2">
-        <v>2975</v>
+        <v>21</v>
       </c>
       <c r="E3" s="3">
-        <f>D3/B3</f>
-        <v>1.1535478867778208</v>
+        <f t="shared" ref="E3:E33" si="0">D3/B3</f>
+        <v>1.1052631578947369</v>
       </c>
       <c r="F3" s="2">
-        <v>4514</v>
+        <v>0</v>
       </c>
       <c r="G3" s="2">
-        <v>3313</v>
+        <v>21</v>
       </c>
       <c r="H3" s="3">
-        <f>G3/B3</f>
-        <v>1.2846064366033347</v>
+        <f t="shared" ref="H3:H33" si="1">G3/B3</f>
+        <v>1.1052631578947369</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2">
-        <v>33523</v>
+        <v>291</v>
       </c>
       <c r="C4" s="2">
         <v>0</v>
       </c>
       <c r="D4" s="2">
-        <v>37928</v>
+        <v>291</v>
       </c>
       <c r="E4" s="3">
-        <f t="shared" ref="E4:E33" si="0">D4/B4</f>
-        <v>1.1314023207946782</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="F4" s="2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G4" s="2">
-        <v>41190</v>
+        <v>299</v>
       </c>
       <c r="H4" s="3">
-        <f t="shared" ref="H4:H33" si="1">G4/B4</f>
-        <v>1.2287086477940519</v>
+        <f t="shared" si="1"/>
+        <v>1.0274914089347078</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="B5" s="2">
-        <v>9073</v>
+        <v>71</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
       </c>
       <c r="D5" s="2">
-        <v>9962</v>
+        <v>74</v>
       </c>
       <c r="E5" s="3">
         <f t="shared" si="0"/>
-        <v>1.0979830265623278</v>
+        <v>1.0422535211267605</v>
       </c>
       <c r="F5" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" s="2">
-        <v>10341</v>
+        <v>72</v>
       </c>
       <c r="H5" s="3">
         <f t="shared" si="1"/>
-        <v>1.1397553179764135</v>
+        <v>1.0140845070422535</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2">
-        <v>9290</v>
+        <v>2085</v>
       </c>
       <c r="C6" s="2">
         <v>0</v>
       </c>
       <c r="D6" s="2">
-        <v>9962</v>
+        <v>2178</v>
       </c>
       <c r="E6" s="3">
         <f t="shared" si="0"/>
-        <v>1.0723358449946179</v>
+        <v>1.0446043165467627</v>
       </c>
       <c r="F6" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="2">
-        <v>10341</v>
+        <v>2210</v>
       </c>
       <c r="H6" s="3">
         <f t="shared" si="1"/>
-        <v>1.1131324004305705</v>
+        <v>1.0599520383693046</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B7" s="2">
-        <v>7542</v>
+        <v>73</v>
       </c>
       <c r="C7" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2">
-        <v>8181</v>
+        <v>86</v>
       </c>
       <c r="E7" s="3">
         <f t="shared" si="0"/>
-        <v>1.0847255369928401</v>
+        <v>1.178082191780822</v>
       </c>
       <c r="F7" s="2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G7" s="2">
-        <v>9550</v>
+        <v>75</v>
       </c>
       <c r="H7" s="3">
         <f t="shared" si="1"/>
-        <v>1.2662423760275789</v>
+        <v>1.0273972602739727</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2">
-        <v>6105</v>
+        <v>937</v>
       </c>
       <c r="C8" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2">
-        <v>7049</v>
+        <v>965</v>
       </c>
       <c r="E8" s="3">
         <f t="shared" si="0"/>
-        <v>1.1546273546273547</v>
+        <v>1.0298826040554963</v>
       </c>
       <c r="F8" s="2">
-        <v>234</v>
+        <v>0</v>
       </c>
       <c r="G8" s="2">
-        <v>7906</v>
+        <v>1102</v>
       </c>
       <c r="H8" s="3">
         <f t="shared" si="1"/>
-        <v>1.2950040950040951</v>
+        <v>1.176093916755603</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B9" s="2">
-        <v>6527</v>
+        <v>9073</v>
       </c>
       <c r="C9" s="2">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="D9" s="2">
-        <v>7213</v>
+        <v>9962</v>
       </c>
       <c r="E9" s="3">
         <f t="shared" si="0"/>
-        <v>1.105101884479853</v>
+        <v>1.0979830265623278</v>
       </c>
       <c r="F9" s="2">
-        <v>416</v>
+        <v>2</v>
       </c>
       <c r="G9" s="2">
-        <v>8140</v>
+        <v>10341</v>
       </c>
       <c r="H9" s="3">
         <f t="shared" si="1"/>
-        <v>1.24712731729738</v>
+        <v>1.1397553179764135</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B10" s="2">
-        <v>629</v>
+        <v>9290</v>
       </c>
       <c r="C10" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D10" s="2">
-        <v>746</v>
+        <v>9962</v>
       </c>
       <c r="E10" s="3">
         <f t="shared" si="0"/>
-        <v>1.1860095389507155</v>
+        <v>1.0723358449946179</v>
       </c>
       <c r="F10" s="2">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="G10" s="2">
-        <v>822</v>
+        <v>10341</v>
       </c>
       <c r="H10" s="3">
         <f t="shared" si="1"/>
-        <v>1.3068362480127187</v>
+        <v>1.1131324004305705</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="B11" s="2">
-        <v>426</v>
+        <v>33523</v>
       </c>
       <c r="C11" s="2">
         <v>0</v>
       </c>
       <c r="D11" s="2">
-        <v>482</v>
+        <v>37928</v>
       </c>
       <c r="E11" s="3">
         <f t="shared" si="0"/>
-        <v>1.1314553990610328</v>
+        <v>1.1314023207946782</v>
       </c>
       <c r="F11" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G11" s="2">
-        <v>556</v>
+        <v>41190</v>
       </c>
       <c r="H11" s="3">
         <f t="shared" si="1"/>
-        <v>1.3051643192488263</v>
+        <v>1.2287086477940519</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12" s="2">
-        <v>538</v>
+        <v>426</v>
       </c>
       <c r="C12" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="2">
-        <v>608</v>
+        <v>482</v>
       </c>
       <c r="E12" s="3">
         <f t="shared" si="0"/>
-        <v>1.1301115241635689</v>
+        <v>1.1314553990610328</v>
       </c>
       <c r="F12" s="2">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="G12" s="2">
-        <v>674</v>
+        <v>556</v>
       </c>
       <c r="H12" s="3">
         <f t="shared" si="1"/>
-        <v>1.2527881040892193</v>
+        <v>1.3051643192488263</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B13" s="2">
-        <v>19</v>
+        <v>7542</v>
       </c>
       <c r="C13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13" s="2">
-        <v>21</v>
+        <v>8181</v>
       </c>
       <c r="E13" s="3">
         <f t="shared" si="0"/>
-        <v>1.1052631578947369</v>
+        <v>1.0847255369928401</v>
       </c>
       <c r="F13" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G13" s="2">
-        <v>21</v>
+        <v>9550</v>
       </c>
       <c r="H13" s="3">
         <f t="shared" si="1"/>
-        <v>1.1052631578947369</v>
+        <v>1.2662423760275789</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="B14" s="2">
-        <v>937</v>
+        <v>675</v>
       </c>
       <c r="C14" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2">
-        <v>965</v>
+        <v>796</v>
       </c>
       <c r="E14" s="3">
         <f t="shared" si="0"/>
-        <v>1.0298826040554963</v>
+        <v>1.1792592592592592</v>
       </c>
       <c r="F14" s="2">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G14" s="2">
-        <v>1102</v>
+        <v>862</v>
       </c>
       <c r="H14" s="3">
         <f t="shared" si="1"/>
-        <v>1.176093916755603</v>
+        <v>1.277037037037037</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B15" s="2">
-        <v>1667</v>
+        <v>538</v>
       </c>
       <c r="C15" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D15" s="2">
-        <v>1836</v>
+        <v>608</v>
       </c>
       <c r="E15" s="3">
         <f t="shared" si="0"/>
-        <v>1.101379724055189</v>
+        <v>1.1301115241635689</v>
       </c>
       <c r="F15" s="2">
-        <v>169</v>
+        <v>29</v>
       </c>
       <c r="G15" s="2">
-        <v>2101</v>
+        <v>674</v>
       </c>
       <c r="H15" s="3">
         <f t="shared" si="1"/>
-        <v>1.2603479304139171</v>
+        <v>1.2527881040892193</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="B16" s="2">
-        <v>2085</v>
+        <v>108159</v>
       </c>
       <c r="C16" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="2">
-        <v>2178</v>
+        <v>130921</v>
       </c>
       <c r="E16" s="3">
         <f t="shared" si="0"/>
-        <v>1.0446043165467627</v>
+        <v>1.2104494309303895</v>
       </c>
       <c r="F16" s="2">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G16" s="2">
-        <v>2210</v>
+        <v>142085</v>
       </c>
       <c r="H16" s="3">
         <f t="shared" si="1"/>
-        <v>1.0599520383693046</v>
+        <v>1.3136678408639133</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B17" s="2">
-        <v>533</v>
+        <v>502</v>
       </c>
       <c r="C17" s="2">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D17" s="2">
-        <v>547</v>
+        <v>583</v>
       </c>
       <c r="E17" s="3">
         <f t="shared" si="0"/>
-        <v>1.026266416510319</v>
+        <v>1.1613545816733069</v>
       </c>
       <c r="F17" s="2">
-        <v>1306</v>
+        <v>69</v>
       </c>
       <c r="G17" s="2">
-        <v>588</v>
+        <v>634</v>
       </c>
       <c r="H17" s="3">
         <f t="shared" si="1"/>
-        <v>1.1031894934333959</v>
+        <v>1.2629482071713147</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B18" s="2">
-        <v>3894</v>
+        <v>21282</v>
       </c>
       <c r="C18" s="2">
-        <v>341</v>
+        <v>2</v>
       </c>
       <c r="D18" s="2">
-        <v>3711</v>
+        <v>24698</v>
       </c>
       <c r="E18" s="3">
         <f t="shared" si="0"/>
-        <v>0.95300462249614792</v>
+        <v>1.1605112301475424</v>
       </c>
       <c r="F18" s="2">
-        <v>109900</v>
+        <v>84</v>
       </c>
       <c r="G18" s="2">
-        <v>3967</v>
+        <v>26442</v>
       </c>
       <c r="H18" s="3">
         <f t="shared" si="1"/>
-        <v>1.0187467899332305</v>
+        <v>1.2424584155624472</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B19" s="2">
-        <v>502</v>
+        <v>20749</v>
       </c>
       <c r="C19" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" s="2">
-        <v>583</v>
+        <v>23660</v>
       </c>
       <c r="E19" s="3">
         <f t="shared" si="0"/>
-        <v>1.1613545816733069</v>
+        <v>1.1402959178755603</v>
       </c>
       <c r="F19" s="2">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="G19" s="2">
-        <v>634</v>
+        <v>27130</v>
       </c>
       <c r="H19" s="3">
         <f t="shared" si="1"/>
-        <v>1.2629482071713147</v>
+        <v>1.3075328931514771</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20" s="2">
-        <v>21282</v>
+        <v>21294</v>
       </c>
       <c r="C20" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" s="2">
-        <v>24698</v>
+        <v>24852</v>
       </c>
       <c r="E20" s="3">
         <f t="shared" si="0"/>
-        <v>1.1605112301475424</v>
+        <v>1.1670893209354747</v>
       </c>
       <c r="F20" s="2">
         <v>84</v>
       </c>
       <c r="G20" s="2">
-        <v>26442</v>
+        <v>26002</v>
       </c>
       <c r="H20" s="3">
         <f t="shared" si="1"/>
-        <v>1.2424584155624472</v>
+        <v>1.2210951441720672</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B21" s="2">
-        <v>20749</v>
+        <v>7755</v>
       </c>
       <c r="C21" s="2">
         <v>3</v>
       </c>
       <c r="D21" s="2">
-        <v>23660</v>
+        <v>9424</v>
       </c>
       <c r="E21" s="3">
         <f t="shared" si="0"/>
-        <v>1.1402959178755603</v>
+        <v>1.2152159896840748</v>
       </c>
       <c r="F21" s="2">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G21" s="2">
-        <v>27130</v>
+        <v>10646</v>
       </c>
       <c r="H21" s="3">
         <f t="shared" si="1"/>
-        <v>1.3075328931514771</v>
+        <v>1.3727917472598323</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B22" s="2">
-        <v>21294</v>
+        <v>629</v>
       </c>
       <c r="C22" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" s="2">
-        <v>24852</v>
+        <v>746</v>
       </c>
       <c r="E22" s="3">
         <f t="shared" si="0"/>
-        <v>1.1670893209354747</v>
+        <v>1.1860095389507155</v>
       </c>
       <c r="F22" s="2">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G22" s="2">
-        <v>26002</v>
+        <v>822</v>
       </c>
       <c r="H22" s="3">
         <f t="shared" si="1"/>
-        <v>1.2210951441720672</v>
+        <v>1.3068362480127187</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
@@ -1423,311 +1423,336 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="B24" s="2">
-        <v>291</v>
+        <v>1667</v>
       </c>
       <c r="C24" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D24" s="2">
-        <v>291</v>
+        <v>1836</v>
       </c>
       <c r="E24" s="3">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>1.101379724055189</v>
       </c>
       <c r="F24" s="2">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="G24" s="2">
-        <v>299</v>
+        <v>2101</v>
       </c>
       <c r="H24" s="3">
         <f t="shared" si="1"/>
-        <v>1.0274914089347078</v>
+        <v>1.2603479304139171</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="B25" s="2">
-        <v>19311</v>
+        <v>6105</v>
       </c>
       <c r="C25" s="2">
-        <v>229</v>
+        <v>5</v>
       </c>
       <c r="D25" s="2">
-        <v>17927</v>
+        <v>7049</v>
       </c>
       <c r="E25" s="3">
         <f t="shared" si="0"/>
-        <v>0.92833100305525351</v>
+        <v>1.1546273546273547</v>
       </c>
       <c r="F25" s="2">
-        <v>70952</v>
+        <v>234</v>
       </c>
       <c r="G25" s="2">
-        <v>20958</v>
+        <v>7906</v>
       </c>
       <c r="H25" s="3">
         <f t="shared" si="1"/>
-        <v>1.0852881777225416</v>
+        <v>1.2950040950040951</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="B26" s="2">
-        <v>50778</v>
+        <v>6527</v>
       </c>
       <c r="C26" s="2">
-        <v>132</v>
+        <v>9</v>
       </c>
       <c r="D26" s="2">
-        <v>58950</v>
+        <v>7213</v>
       </c>
       <c r="E26" s="3">
         <f t="shared" si="0"/>
-        <v>1.1609358383551931</v>
+        <v>1.105101884479853</v>
       </c>
       <c r="F26" s="2">
-        <v>29490</v>
+        <v>416</v>
       </c>
       <c r="G26" s="2">
-        <v>68397</v>
+        <v>8140</v>
       </c>
       <c r="H26" s="3">
         <f t="shared" si="1"/>
-        <v>1.3469809760132341</v>
+        <v>1.24712731729738</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="B27" s="2">
-        <v>259045</v>
+        <v>533</v>
       </c>
       <c r="C27" s="2">
-        <v>1196</v>
+        <v>13</v>
       </c>
       <c r="D27" s="2">
-        <v>313745</v>
+        <v>547</v>
       </c>
       <c r="E27" s="3">
         <f t="shared" si="0"/>
-        <v>1.2111602231272558</v>
+        <v>1.026266416510319</v>
       </c>
       <c r="F27" s="2">
-        <v>502354</v>
+        <v>1306</v>
       </c>
       <c r="G27" s="2">
-        <v>347246</v>
+        <v>588</v>
       </c>
       <c r="H27" s="3">
         <f t="shared" si="1"/>
-        <v>1.3404852438765464</v>
+        <v>1.1031894934333959</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B28" s="2">
-        <v>108159</v>
+        <v>3854</v>
       </c>
       <c r="C28" s="2">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D28" s="2">
-        <v>130921</v>
+        <v>4647</v>
       </c>
       <c r="E28" s="3">
         <f t="shared" si="0"/>
-        <v>1.2104494309303895</v>
+        <v>1.2057602490918526</v>
       </c>
       <c r="F28" s="2">
-        <v>29</v>
+        <v>1989</v>
       </c>
       <c r="G28" s="2">
-        <v>142085</v>
+        <v>5122</v>
       </c>
       <c r="H28" s="3">
         <f t="shared" si="1"/>
-        <v>1.3136678408639133</v>
+        <v>1.3290088220031135</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="B29" s="2">
-        <v>7755</v>
+        <v>2579</v>
       </c>
       <c r="C29" s="2">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="D29" s="2">
-        <v>9424</v>
+        <v>2975</v>
       </c>
       <c r="E29" s="3">
         <f t="shared" si="0"/>
-        <v>1.2152159896840748</v>
+        <v>1.1535478867778208</v>
       </c>
       <c r="F29" s="2">
-        <v>84</v>
+        <v>4514</v>
       </c>
       <c r="G29" s="2">
-        <v>10646</v>
+        <v>3313</v>
       </c>
       <c r="H29" s="3">
         <f t="shared" si="1"/>
-        <v>1.3727917472598323</v>
+        <v>1.2846064366033347</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B30" s="2">
-        <v>675</v>
+        <v>50778</v>
       </c>
       <c r="C30" s="2">
-        <v>1</v>
+        <v>132</v>
       </c>
       <c r="D30" s="2">
-        <v>796</v>
+        <v>58950</v>
       </c>
       <c r="E30" s="3">
         <f t="shared" si="0"/>
-        <v>1.1792592592592592</v>
+        <v>1.1609358383551931</v>
       </c>
       <c r="F30" s="2">
-        <v>22</v>
+        <v>29490</v>
       </c>
       <c r="G30" s="2">
-        <v>862</v>
+        <v>68397</v>
       </c>
       <c r="H30" s="3">
         <f t="shared" si="1"/>
-        <v>1.277037037037037</v>
+        <v>1.3469809760132341</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B31" s="2">
-        <v>3854</v>
+        <v>19311</v>
       </c>
       <c r="C31" s="2">
-        <v>20</v>
+        <v>229</v>
       </c>
       <c r="D31" s="2">
-        <v>4647</v>
+        <v>17927</v>
       </c>
       <c r="E31" s="3">
         <f t="shared" si="0"/>
-        <v>1.2057602490918526</v>
+        <v>0.92833100305525351</v>
       </c>
       <c r="F31" s="2">
-        <v>1989</v>
+        <v>70952</v>
       </c>
       <c r="G31" s="2">
-        <v>5122</v>
+        <v>20958</v>
       </c>
       <c r="H31" s="3">
         <f t="shared" si="1"/>
-        <v>1.3290088220031135</v>
+        <v>1.0852881777225416</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="B32" s="2">
-        <v>71</v>
+        <v>3894</v>
       </c>
       <c r="C32" s="2">
-        <v>0</v>
+        <v>341</v>
       </c>
       <c r="D32" s="2">
-        <v>74</v>
+        <v>3711</v>
       </c>
       <c r="E32" s="3">
         <f t="shared" si="0"/>
-        <v>1.0422535211267605</v>
+        <v>0.95300462249614792</v>
       </c>
       <c r="F32" s="2">
-        <v>0</v>
+        <v>109900</v>
       </c>
       <c r="G32" s="2">
-        <v>72</v>
+        <v>3967</v>
       </c>
       <c r="H32" s="3">
         <f t="shared" si="1"/>
-        <v>1.0140845070422535</v>
+        <v>1.0187467899332305</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B33" s="2">
-        <v>73</v>
+        <v>259045</v>
       </c>
       <c r="C33" s="2">
-        <v>0</v>
+        <v>1196</v>
       </c>
       <c r="D33" s="2">
-        <v>86</v>
+        <v>313745</v>
       </c>
       <c r="E33" s="3">
         <f t="shared" si="0"/>
-        <v>1.178082191780822</v>
+        <v>1.2111602231272558</v>
       </c>
       <c r="F33" s="2">
-        <v>2</v>
+        <v>502354</v>
       </c>
       <c r="G33" s="2">
-        <v>75</v>
+        <v>347246</v>
       </c>
       <c r="H33" s="3">
         <f t="shared" si="1"/>
-        <v>1.0273972602739727</v>
+        <v>1.3404852438765464</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B34" s="5"/>
+        <v>48</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>5</v>
+      </c>
       <c r="C34" s="6">
-        <f>AVERAGE(E3:E33)</f>
-        <v>1.11761803703935</v>
+        <f>AVERAGE(C3:C33)</f>
+        <v>64.645161290322577</v>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
       <c r="F34" s="6">
-        <f>AVERAGE(H3:H33)</f>
-        <v>1.2143778281984563</v>
+        <f>AVERAGE(F3:F33)</f>
+        <v>23291.032258064515</v>
       </c>
       <c r="G34" s="5"/>
       <c r="H34" s="5"/>
     </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35" s="5"/>
+      <c r="B35" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" s="6">
+        <f>AVERAGE(E4:E34)</f>
+        <v>1.1180298663441703</v>
+      </c>
+      <c r="D35" s="5"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="6">
+        <f>AVERAGE(H4:H34)</f>
+        <v>1.2180149838752463</v>
+      </c>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:H33">
+    <sortCondition ref="F3:F33"/>
+  </sortState>
+  <mergeCells count="9">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A34:B34"/>
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="F34:H34"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="F35:H35"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Remove datasets that result in ratio less than 1.0, and regenerate output files.
</commit_message>
<xml_diff>
--- a/resource/result.xlsx
+++ b/resource/result.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_Files\_Lessons\ALGORITHM\Project\resource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14622D44-2112-4698-B9D1-C7263E7E6A14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B51F813-F251-46DF-93E0-3CF12D1D0C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5130" yWindow="2760" windowWidth="19200" windowHeight="11170" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EXACT" sheetId="9" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="48">
   <si>
     <t>att48</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -137,10 +137,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>gr666</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>gr96</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -158,10 +154,6 @@
   </si>
   <si>
     <t>lin105</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>pa561</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -612,35 +604,35 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E1" s="5"/>
       <c r="F1" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G1" s="5"/>
       <c r="H1" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I1" s="5"/>
       <c r="J1" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>5</v>
@@ -661,7 +653,7 @@
         <v>6</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -728,7 +720,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B5" s="2">
         <v>71</v>
@@ -785,7 +777,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{260DB66E-1FFD-4D32-BA5D-DB6972467A37}">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" style="1" customWidth="1"/>
@@ -795,7 +787,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>4</v>
@@ -847,7 +839,7 @@
         <v>21</v>
       </c>
       <c r="E3" s="3">
-        <f t="shared" ref="E3:E33" si="0">D3/B3</f>
+        <f t="shared" ref="E3:E31" si="0">D3/B3</f>
         <v>1.1052631578947369</v>
       </c>
       <c r="F3" s="2">
@@ -857,7 +849,7 @@
         <v>21</v>
       </c>
       <c r="H3" s="3">
-        <f t="shared" ref="H3:H33" si="1">G3/B3</f>
+        <f t="shared" ref="H3:H31" si="1">G3/B3</f>
         <v>1.1052631578947369</v>
       </c>
     </row>
@@ -891,7 +883,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B5" s="2">
         <v>71</v>
@@ -947,7 +939,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B7" s="2">
         <v>73</v>
@@ -1143,7 +1135,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B14" s="2">
         <v>675</v>
@@ -1199,7 +1191,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B16" s="2">
         <v>108159</v>
@@ -1227,7 +1219,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" s="2">
         <v>502</v>
@@ -1255,7 +1247,7 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B18" s="2">
         <v>21282</v>
@@ -1283,7 +1275,7 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B19" s="2">
         <v>20749</v>
@@ -1311,7 +1303,7 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B20" s="2">
         <v>21294</v>
@@ -1339,7 +1331,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B21" s="2">
         <v>7755</v>
@@ -1395,7 +1387,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B23" s="2">
         <v>14379</v>
@@ -1535,7 +1527,7 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B28" s="2">
         <v>3854</v>
@@ -1591,7 +1583,7 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B30" s="2">
         <v>50778</v>
@@ -1622,137 +1614,81 @@
         <v>31</v>
       </c>
       <c r="B31" s="2">
-        <v>19311</v>
+        <v>259045</v>
       </c>
       <c r="C31" s="2">
-        <v>229</v>
+        <v>1196</v>
       </c>
       <c r="D31" s="2">
-        <v>17927</v>
+        <v>313745</v>
       </c>
       <c r="E31" s="3">
         <f t="shared" si="0"/>
-        <v>0.92833100305525351</v>
+        <v>1.2111602231272558</v>
       </c>
       <c r="F31" s="2">
-        <v>70952</v>
+        <v>502354</v>
       </c>
       <c r="G31" s="2">
-        <v>20958</v>
+        <v>347246</v>
       </c>
       <c r="H31" s="3">
         <f t="shared" si="1"/>
-        <v>1.0852881777225416</v>
+        <v>1.3404852438765464</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B32" s="2">
-        <v>3894</v>
-      </c>
-      <c r="C32" s="2">
-        <v>341</v>
-      </c>
-      <c r="D32" s="2">
-        <v>3711</v>
-      </c>
-      <c r="E32" s="3">
-        <f t="shared" si="0"/>
-        <v>0.95300462249614792</v>
-      </c>
-      <c r="F32" s="2">
-        <v>109900</v>
-      </c>
-      <c r="G32" s="2">
-        <v>3967</v>
-      </c>
-      <c r="H32" s="3">
-        <f t="shared" si="1"/>
-        <v>1.0187467899332305</v>
-      </c>
+      <c r="A32" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C32" s="6">
+        <f>AVERAGE(C3:C31)</f>
+        <v>49.448275862068968</v>
+      </c>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="6">
+        <f>AVERAGE(F3:F31)</f>
+        <v>18661.03448275862</v>
+      </c>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B33" s="2">
-        <v>259045</v>
-      </c>
-      <c r="C33" s="2">
-        <v>1196</v>
-      </c>
-      <c r="D33" s="2">
-        <v>313745</v>
-      </c>
-      <c r="E33" s="3">
-        <f t="shared" si="0"/>
-        <v>1.2111602231272558</v>
-      </c>
-      <c r="F33" s="2">
-        <v>502354</v>
-      </c>
-      <c r="G33" s="2">
-        <v>347246</v>
-      </c>
-      <c r="H33" s="3">
-        <f t="shared" si="1"/>
-        <v>1.3404852438765464</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A34" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C34" s="6">
-        <f>AVERAGE(C3:C33)</f>
-        <v>64.645161290322577</v>
-      </c>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="6">
-        <f>AVERAGE(F3:F33)</f>
-        <v>23291.032258064515</v>
-      </c>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A35" s="5"/>
-      <c r="B35" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C35" s="6">
-        <f>AVERAGE(E4:E34)</f>
-        <v>1.1180298663441703</v>
-      </c>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="6">
-        <f>AVERAGE(H4:H34)</f>
-        <v>1.2180149838752463</v>
-      </c>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
+      <c r="A33" s="5"/>
+      <c r="B33" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C33" s="6">
+        <f>AVERAGE(E4:E32)</f>
+        <v>1.1306985844562039</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="6">
+        <f>AVERAGE(H4:H32)</f>
+        <v>1.2298719481643434</v>
+      </c>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:H33">
-    <sortCondition ref="F3:F33"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:H31">
+    <sortCondition ref="F3:F31"/>
   </sortState>
   <mergeCells count="9">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="F34:H34"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="F35:H35"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="F33:H33"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>